<commit_message>
🔧 Improve scheduler to detect race tomorrow and conditionally run predictions
- scheduler.py now outputs RACE_TOMORROW flag and race details
- Workflow only runs data fetching & commit when a race is tomorrow
- Reduces unnecessary CI runs on non-race days
- Prevents empty artifact uploads and failed commits

Changes:
- scheduler.py: Output RACE_TAG, RACE_DATE, RACE_VENUE, RACE_TOMORROW
- predict-schedule.yml: Use job outputs to conditionally run upload/commit steps
  - Check-race step parses scheduler output for environment variables
  - Upload and commit steps now only execute if race_tomorrow == 'true'
</commit_message>
<xml_diff>
--- a/data/results/2026-04-06_ST.xlsx
+++ b/data/results/2026-04-06_ST.xlsx
@@ -19,6 +19,7 @@
     <sheet name="R9" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="R10" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="R11" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Dividends" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -15845,6 +15846,1950 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D107"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>race_no</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>bet_type</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>combo</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>dividend</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>231.5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1,12</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>quinella</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1,12</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>12,1</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>tierce</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>12,1,9</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>3616</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1,9,12</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>first4</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1,9,12,14</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>quartet</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>12,1,9,14</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>24545</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>66.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>24.5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>1,14</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>quinella</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>1,14</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>542.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>14,1</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>959</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>tierce</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>14,1,10</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>39585</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>1,10,14</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>5917</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>2</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>first4</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>1,8,10,14</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>6007</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>quartet</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>14,1,10,8</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>256411</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>132.5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>39.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>7,8</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>3</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>quinella</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>7,8</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>683</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>3</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>7,8</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1529</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>3</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>tierce</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>7,8,1</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>6991</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>3</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>1,7,8</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1062</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>3</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>1,10,14/1,7,8</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>859503</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>3</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>first4</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>1,3,7,8</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>1216</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>3</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>quartet</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>7,8,1,3</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>46159</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>4</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>146.5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>4</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>4</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>3,14</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>4</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>quinella</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>3,14</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>4</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>14,3</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>1385</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>4</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>tierce</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>14,3,9</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>58061</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>4</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>3,9,14</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>11124</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>4</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>first4</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>3,9,12,14</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>72771</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>4</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>quartet</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>14,3,9,12</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>535388</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>5</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>5</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>5</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>3,14</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>155.5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>5</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>quinella</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>3,14</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>5</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>3,14</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>1464</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>5</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>tierce</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>3,14,6</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>12431</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>5</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>3,6,14</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>1834</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>5</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>3,9,14/3,6,14</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>1099880</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>5</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>first4</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>3,6,7,14</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>1038</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>5</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>quartet</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>3,14,6,7</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>41441</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>6</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>50.5</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>6</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>6</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>1,4</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>6</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>quinella</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>1,4</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>6</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>4,1</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>6</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>tierce</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>4,1,12</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>1175</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>6</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>1,4,12</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>6</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>first4</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>1,4,5,12</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>6</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>quartet</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>4,1,12,5</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>8328</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>7</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>7</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>10.1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>7</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>1,2</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>10.5</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>7</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>quinella</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>1,2</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>14.5</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>7</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>1,2</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>7</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>tierce</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>7</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>1,2,3</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>7</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>1,4,12/1,2,3</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>7</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>3,6,14/1,4,12/1,2,3</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>115387</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>7</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>3,6,14/1,4,12/Any Combination</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>2307</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>7</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>first4</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>1,2,3,6</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>7</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>quartet</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>1,2,3,6</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>8</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>55.5</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>8</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>8</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2,4</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>42.5</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>8</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>quinella</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2,4</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>131.5</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>8</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2,4</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>8</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>tierce</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>2,4,6</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>8</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>2,4,6</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>8</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>first4</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>2,4,6,8</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>8</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>quartet</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>2,4,6,8</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>1444</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>9</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>39.5</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>9</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>14.5</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>9</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>3,8</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>28.5</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>9</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>quinella</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>3,8</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>63.5</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>9</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>3,8</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>9</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>tierce</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>3,8,1</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>9</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>1,3,8</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>9</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>2,4,6/1,3,8</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>1035</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>9</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>first4</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>1,3,6,8</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>9</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>quartet</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>3,8,1,6</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>5507</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>10</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>440.5</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>10</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>79.5</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>10</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>4,6</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>10</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>quinella</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>4,6</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>666</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>10</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>6,4</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>1655</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>10</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>tierce</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>6,4,8</t>
+        </is>
+      </c>
+      <c r="D94" t="n">
+        <v>3973</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>10</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>4,6,8</t>
+        </is>
+      </c>
+      <c r="D95" t="n">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>10</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>first4</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>1,4,6,8</t>
+        </is>
+      </c>
+      <c r="D96" t="n">
+        <v>662</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>10</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>quartet</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>6,4,8,1</t>
+        </is>
+      </c>
+      <c r="D97" t="n">
+        <v>32656</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>11</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>win</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D98" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>11</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D99" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>11</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>place</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>3,4</t>
+        </is>
+      </c>
+      <c r="D100" t="n">
+        <v>85.5</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>11</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>quinella</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>3,4</t>
+        </is>
+      </c>
+      <c r="D101" t="n">
+        <v>250.5</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>11</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>forecast</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>4,3</t>
+        </is>
+      </c>
+      <c r="D102" t="n">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>11</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>tierce</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>4,3,9</t>
+        </is>
+      </c>
+      <c r="D103" t="n">
+        <v>6937</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>11</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>3,4,9</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>11</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>trio</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>4,6,8/3,4,9</t>
+        </is>
+      </c>
+      <c r="D105" t="n">
+        <v>67357</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>11</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>first4</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>3,4,9,11</t>
+        </is>
+      </c>
+      <c r="D106" t="n">
+        <v>3802</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>11</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>quartet</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>4,3,9,11</t>
+        </is>
+      </c>
+      <c r="D107" t="n">
+        <v>68729</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>